<commit_message>
Plan de carga v2: numeros reais da DevSales (GAPCHECK 12/08)
- Fila 0 nova: deploy do manifest como pre-requisito (campos do fluxo
  nao existem na DevSales; nativos ProductCode/StockKeepingUnit avaliados
  e descartados por nao poderem ser unico+External ID)
- Kits: reutilizar tipo existente Bundle->BundleComponent
  (0yoao0000019FldAAE); campos reais MainProductRoleCat/AssociatedProductRoleCat
- Vehicle: VIN confirmado (VehicleIdentificationNumber); sem lookup nativo
  a Location - decisao aberta aguardando GAPCHECK3 (Asset.LocationId)
- Contagens: 250 Product2 (3 sem entrada Standard), 224 VehicleDefinition
  (0 orfas), 6 Vehicle, 20 Location, 2 Pricebook2, 0 kits, 0 search config;
  moedas USD/CRC

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012ouMFEvRtMPEA2sZAxeatj
</commit_message>
<xml_diff>
--- a/docs/carga/Carga_Productos_Precios_Inventario.xlsx
+++ b/docs/carga/Carga_Productos_Precios_Inventario.xlsx
@@ -228,460 +228,502 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">0</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Location</t>
+          <t xml:space="preserve">(pré-requisito) Deploy do manifest</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Centros/sucursales físicos. Ancla del inventario de vehículos y del Vehicle Inventory Search (búsqueda multi-tienda).</t>
+          <t xml:space="preserve">Os campos que os fluxos consomem NÃO são carga de dados: chegam por deploy do manifest mestre (package-venta-guiada-completo.xml) na org destino.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Name, LocationType, ExternalReference, IsInventoryLocation=true</t>
+          <t xml:space="preserve">QuoteLineItem.AvailabilityStatus__c/AvailabilityDetail__c, Order.SapStatus__c/SapOrderNumber__c/SapInvoiceNumber__c/SapInvoiceDate__c, Product2.SapMaterialCode__c + classes/LWC/flows</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ExternalReference = código del centro (WERKS)</t>
+          <t xml:space="preserve">n/a (metadata, não dados)</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">T001W (centros/plantas)</t>
+          <t xml:space="preserve">n/a</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Decenas · carga única + mantenimiento</t>
+          <t xml:space="preserve">1 deploy</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PENDIENTE T09: lista oficial de centros del GrupoQ. Sin Location no hay búsqueda por ubicación ni traslados (US-037).</t>
+          <t xml:space="preserve">GAPCHECK 12/08 na DevSales: esses campos ainda NÃO existem lá. Nativos avaliados antes de criar: ProductCode e StockKeepingUnit existem no Product2, mas nenhum pode ser único + External ID — a garantia anti-duplicado do banco exige o campo custom.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pricebook2</t>
+          <t xml:space="preserve">Location</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Una lista de precios por sociedad/canal (p.ej. C101-Q1, C105-Q1, N101-Q1, N105-Q1). La Standard ya existe en la org.</t>
+          <t xml:space="preserve">Centros/sucursales físicos. Ancla del inventario de vehículos y del Vehicle Inventory Search (búsqueda multi-tienda).</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Name, IsActive, Description</t>
+          <t xml:space="preserve">Name, LocationType, ExternalReference, IsInventoryLocation=true</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Name (convención sociedad-canal)</t>
+          <t xml:space="preserve">ExternalReference = código del centro (WERKS)</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Estructura comercial (org. de ventas / canal de distribución)</t>
+          <t xml:space="preserve">T001W (centros/plantas)</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unidades · carga única</t>
+          <t xml:space="preserve">DevSales: 20 ya cargadas · carga única + mantenimiento</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">La moneda NO vive en la lista: vive en cada PricebookEntry (org multi-moneda).</t>
+          <t xml:space="preserve">Validar las 20 existentes contra la lista oficial de centros del GrupoQ (T09). Sin Location no hay búsqueda por ubicación ni traslados (US-037).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Product2</t>
+          <t xml:space="preserve">Pricebook2</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Catálogo completo: vehículos, repuestos (ZREP), accesorios y P&amp;A. Base de TODO el flujo guiado.</t>
+          <t xml:space="preserve">Una lista de precios por sociedad/canal (p.ej. C101-Q1, C105-Q1, N101-Q1, N105-Q1). La Standard ya existe en la org.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Name, ProductCode, SapMaterialCode__c, IsActive, Family, Description</t>
+          <t xml:space="preserve">Name, IsActive, Description</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SapMaterialCode__c (único + External ID → upsert idempotente y a prueba de duplicados)</t>
+          <t xml:space="preserve">Name (convención sociedad-canal)</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARA + MVKE (maestro de materiales por sociedad/canal) vía réplica Mule</t>
+          <t xml:space="preserve">Estructura comercial (org. de ventas / canal de distribución)</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Miles · carga inicial + delta diario/near-real-time</t>
+          <t xml:space="preserve">DevSales: solo 2 hoy (Standard + 1) — faltan las listas por sociedad/canal</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Backfill obligatorio: SapMaterialCode__c = MATNR también en los legados. Family distingue Vehículo / Repuesto / Accesorio (StandardValueSet Product2Family ya en el manifest).</t>
+          <t xml:space="preserve">La moneda NO vive en la lista: vive en cada PricebookEntry. Monedas activas de la org: USD y CRC (GAPCHECK).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">4</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PricebookEntry (Standard)</t>
+          <t xml:space="preserve">Product2</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Entrada en la lista Standard — OBLIGATORIA antes de cualquier lista custom (regla de la plataforma).</t>
+          <t xml:space="preserve">Catálogo completo: vehículos, repuestos (ZREP), accesorios y P&amp;A. Base de TODO el flujo guiado.</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pricebook2Id (Std), Product2Id, UnitPrice, CurrencyIsoCode, IsActive</t>
+          <t xml:space="preserve">Name, ProductCode, SapMaterialCode__c, IsActive, Family, Description</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No hay external id nativo: cargar por Data Loader relacionando Product2 vía SapMaterialCode__c</t>
+          <t xml:space="preserve">SapMaterialCode__c (único + External ID → upsert idempotente y a prueba de duplicados)</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Condición de precio de lista (ZGQREF / precio base)</t>
+          <t xml:space="preserve">MARA + MVKE (maestro de materiales por sociedad/canal) vía réplica Mule</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">= productos × monedas</t>
+          <t xml:space="preserve">DevSales: 250 activos hoy · carga inicial + delta diario/near-real-time</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sin la entrada Standard, el insert en la lista custom FALLA. Orden de carga: siempre después de Product2.</t>
+          <t xml:space="preserve">SapMaterialCode__c llega por el deploy (fila 0); backfill = MATNR también en los 250 existentes. Family distingue Vehículo / Repuesto / Accesorio (StandardValueSet Product2Family ya en el manifest).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">5</t>
+          <t xml:space="preserve">4</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PricebookEntry (listas sociedad/canal)</t>
+          <t xml:space="preserve">PricebookEntry (Standard)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Precio vigente por lista comercial.</t>
+          <t xml:space="preserve">Entrada en la lista Standard — OBLIGATORIA antes de cualquier lista custom (regla de la plataforma).</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">+ UseStandardPrice=false</t>
+          <t xml:space="preserve">Pricebook2Id (Std), Product2Id, UnitPrice, CurrencyIsoCode, IsActive</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ídem fila 4</t>
+          <t xml:space="preserve">No hay external id nativo: cargar por Data Loader relacionando Product2 vía SapMaterialCode__c</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Condiciones por org. de ventas/canal</t>
+          <t xml:space="preserve">Condición de precio de lista (ZGQREF / precio base)</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">= productos × listas</t>
+          <t xml:space="preserve">= productos × monedas (USD, CRC)</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Para repuestos el precio AUTORITATIVO en la cotización sigue siendo SAP (consulta viva); la lista local es el soporte del modelo nativo (toda QuoteLineItem apunta a un PricebookEntry). Pricing/descuentos = US-024/025/066/092; vigencia = US-103.</t>
+          <t xml:space="preserve">Sin la entrada Standard, el insert en la lista custom FALLA. GAPCHECK: hay 3 productos activos SIN entrada Standard hoy — corregirlos antes de cargar listas custom.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">6</t>
+          <t xml:space="preserve">5</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ProductRelationshipType</t>
+          <t xml:space="preserve">PricebookEntry (listas sociedad/canal)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tipo del vínculo kit→componente. Prerrequisito del ProductRelatedComponent.</t>
+          <t xml:space="preserve">Precio vigente por lista comercial.</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Name, MainProductRole, AssociatedProductRole</t>
+          <t xml:space="preserve">+ UseStandardPrice=false</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">n/a (1 registro)</t>
+          <t xml:space="preserve">ídem fila 4</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">n/a</t>
+          <t xml:space="preserve">Condiciones por org. de ventas/canal</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 registro</t>
+          <t xml:space="preserve">= productos × listas</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Verificar valores de picklist disponibles en la org (script GAP).</t>
+          <t xml:space="preserve">Para repuestos el precio AUTORITATIVO en la cotización sigue siendo SAP (consulta viva); la lista local es el soporte del modelo nativo (toda QuoteLineItem apunta a un PricebookEntry). Pricing/descuentos = US-024/025/066/092; vigencia = US-103.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">7</t>
+          <t xml:space="preserve">6</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ProductRelatedComponent</t>
+          <t xml:space="preserve">ProductRelationshipType</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kits/combos/agrupaciones (GQ-PV-02-029). El grid ya expande y renderiza componentes.</t>
+          <t xml:space="preserve">Tipo del vínculo kit→componente. Prerrequisito del ProductRelatedComponent.</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ParentProductId, ChildProductId, Quantity, ProductRelationshipTypeId</t>
+          <t xml:space="preserve">NADA A CARGAR: reutilizar el registro existente "Bundle to Bundle Component Relationship" (Bundle → BundleComponent)</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Parent+Child resueltos vía SapMaterialCode__c de ambos lados</t>
+          <t xml:space="preserve">Id existente en DevSales: 0yoao0000019FldAAE</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">BOM comercial / listas técnicas del DBM</t>
+          <t xml:space="preserve">n/a</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Centenas</t>
+          <t xml:space="preserve">0 (ya existen 4 tipos)</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Objeto confirmado habilitado en DevSales (12/08).</t>
+          <t xml:space="preserve">GAPCHECK: los campos reales son MainProductRoleCat / AssociatedProductRoleCat (no MainProductRole). Valores: Bundle, Set, AddOn, ProductRequest → BundleComponent, SetComponent, AddOnComponent...</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">8</t>
+          <t xml:space="preserve">7</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">VehicleDefinition</t>
+          <t xml:space="preserve">ProductRelatedComponent</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Modelo/versión (ficha técnica) de cada Product2 de vehículo. Cadena oficial: VehicleDefinition.ProductId → Product2.</t>
+          <t xml:space="preserve">Kits/combos/agrupaciones (GQ-PV-02-029). El grid ya expande y renderiza componentes.</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Name, ProductId, atributos del modelo (marca, carrocería, transmisión, año...)</t>
+          <t xml:space="preserve">ParentProductId, ChildProductId, Quantity, ProductRelationshipTypeId</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ProductId (1:1 con el Product2 del vehículo)</t>
+          <t xml:space="preserve">Parent+Child resueltos vía SapMaterialCode__c de ambos lados</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Maestro de modelos del DBM (VELO/VLC)</t>
+          <t xml:space="preserve">BOM comercial / listas técnicas del DBM</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Centenas</t>
+          <t xml:space="preserve">DevSales: 0 hoy · centenas al cargar</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Base del Inventory Search: VehicleSearchableField apunta a campos de aquí. OJO: VehicleDefinitions con ProductId nulo rompen subqueries (bug 3 de la suite) — cargar SIEMPRE con ProductId.</t>
+          <t xml:space="preserve">Objeto habilitado y confirmado (12/08); ProductRelationshipTypeId = 0yoao0000019FldAAE en todos los registros.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">9</t>
+          <t xml:space="preserve">8</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vehicle</t>
+          <t xml:space="preserve">VehicleDefinition</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Inventario PROPIO de vehículos: cada unidad física con VIN. Cadena: Vehicle.VehicleDefinitionId → VehicleDefinition; Vehicle.AssetId → Asset al vender.</t>
+          <t xml:space="preserve">Modelo/versión (ficha técnica) de cada Product2 de vehículo. Cadena oficial: VehicleDefinition.ProductId → Product2.</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Name, VehicleDefinitionId, VIN, Status, LocationId (verificar API name con el script GAP)</t>
+          <t xml:space="preserve">Name, ProductId, atributos del modelo (marca, carrocería, transmisión, año...)</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">VIN (único en la org)</t>
+          <t xml:space="preserve">ProductId (1:1 con el Product2 del vehículo)</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stock de vehículos del DBM (VLC) por centro</t>
+          <t xml:space="preserve">Maestro de modelos del DBM (VELO/VLC)</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Miles · delta por movimiento (ingreso/venta/traslado)</t>
+          <t xml:space="preserve">DevSales: 224 hoy (0 huérfanas — GAPCHECK)</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Usados: entran por HU-045 (Appraisal → Vehicle). LocationId liga la unidad al centro para la búsqueda multi-tienda.</t>
+          <t xml:space="preserve">Base del Inventory Search: VehicleSearchableField apunta a campos de aquí. OJO: VehicleDefinitions con ProductId nulo rompen subqueries (bug 3 de la suite) — cargar SIEMPRE con ProductId.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">10</t>
+          <t xml:space="preserve">9</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Asset</t>
+          <t xml:space="preserve">Vehicle</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vehículo VENDIDO/entregado — relación cliente↔vehículo para posventa. Asset.Product2Id → Product2.</t>
+          <t xml:space="preserve">Inventario PROPIO de vehículos: cada unidad física con VIN. Cadena: Vehicle.VehicleDefinitionId → VehicleDefinition; Vehicle.AssetId → Asset al vender.</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">AccountId, Product2Id, SerialNumber=VIN, Status, PurchaseDate</t>
+          <t xml:space="preserve">Name, VehicleDefinitionId, VehicleIdentificationNumber (VIN — API name confirmado), Status + vínculo con el centro (DECISIÓN ABIERTA)</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SerialNumber + AccountId</t>
+          <t xml:space="preserve">VehicleIdentificationNumber (único en la org)</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Histórico de ventas del DBM</t>
+          <t xml:space="preserve">Stock de vehículos del DBM (VLC) por centro</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Miles (histórico retroactivo)</t>
+          <t xml:space="preserve">DevSales: 6 hoy · miles al cargar · delta por movimiento</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">El flujo NUEVO ya lo crea solo (Order_Facturado_Handler al facturar). La carga aquí es únicamente el histórico anterior al go-live.</t>
+          <t xml:space="preserve">GAPCHECK: Vehicle NO tiene lookup nativo a Location — solo el campo compuesto de dirección (Location ADDRESS). Candidato nativo por verificar: Asset.LocationId (GAPCHECK3); si tampoco existe, crear lookup custom Vehicle → Location (única creación de campo de todo el plan).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">10</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Asset</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vehículo VENDIDO/entregado — relación cliente↔vehículo para posventa. Asset.Product2Id → Product2.</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AccountId, Product2Id, SerialNumber=VIN, Status, PurchaseDate</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SerialNumber + AccountId</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Histórico de ventas del DBM</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Miles (histórico retroactivo)</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El flujo NUEVO ya lo crea solo (Order_Facturado_Handler al facturar). La carga aquí es únicamente el histórico anterior al go-live.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">11</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">VehicleSearchableField (setup)</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Configuración del Vehicle Inventory Search: qué campos son criterio, cuáles se muestran, ordenan y agregan.</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Es CONFIGURACIÓN (Setup), no carga de datos</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">n/a</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">n/a</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Decenas de campos</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DevSales: 0 (búsqueda SIN configurar)</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Configurar DESPUÉS de cargar VehicleDefinition + Vehicle + Location, y probar la búsqueda con datos reales.</t>
         </is>

</xml_diff>

<commit_message>
Plan de carga v3: vinculo Vehicle-centro fechado via Asset.LocationId (nativo, zero campos novos)
GAPCHECK3 confirmou Asset.LocationId (REFERENCE -> Location); Asset passa
a vir ANTES de Vehicle na ordem de carga (Vehicle.AssetId aponta para ele)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012ouMFEvRtMPEA2sZAxeatj
</commit_message>
<xml_diff>
--- a/docs/carga/Carga_Productos_Precios_Inventario.xlsx
+++ b/docs/carga/Carga_Productos_Precios_Inventario.xlsx
@@ -611,37 +611,37 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vehicle</t>
+          <t xml:space="preserve">Asset</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Inventario PROPIO de vehículos: cada unidad física con VIN. Cadena: Vehicle.VehicleDefinitionId → VehicleDefinition; Vehicle.AssetId → Asset al vender.</t>
+          <t xml:space="preserve">Una fila por UNIDAD física: ancla del vehículo. Asset.Product2Id → Product2 y Asset.LocationId → Location (CENTRO — decisión cerrada por GAPCHECK3). En stock: Account de la propia empresa; al vender: pasa al cliente.</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Name, VehicleDefinitionId, VehicleIdentificationNumber (VIN — API name confirmado), Status + vínculo con el centro (DECISIÓN ABIERTA)</t>
+          <t xml:space="preserve">AccountId (stock: cuenta de la empresa/sucursal), Product2Id, SerialNumber=VIN, Status, LocationId (centro), PurchaseDate (al vender)</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">VehicleIdentificationNumber (único en la org)</t>
+          <t xml:space="preserve">SerialNumber (=VIN)</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stock de vehículos del DBM (VLC) por centro</t>
+          <t xml:space="preserve">Stock de vehículos del DBM (VLC) + histórico de ventas</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DevSales: 6 hoy · miles al cargar · delta por movimiento</t>
+          <t xml:space="preserve">DevSales: 6 hoy · miles al cargar</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GAPCHECK: Vehicle NO tiene lookup nativo a Location — solo el campo compuesto de dirección (Location ADDRESS). Candidato nativo por verificar: Asset.LocationId (GAPCHECK3); si tampoco existe, crear lookup custom Vehicle → Location (única creación de campo de todo el plan).</t>
+          <t xml:space="preserve">DECISIÓN CERRADA (GAPCHECK3 12/08): el vínculo unidad↔centro es Asset.LocationId — NATIVO, cero campos nuevos. Orden: Asset ANTES de Vehicle (Vehicle.AssetId apunta aquí). El flujo nuevo ya crea/actualiza el Asset al facturar (Order_Facturado_Handler); la carga cubre stock actual + histórico.</t>
         </is>
       </c>
     </row>
@@ -653,37 +653,37 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Asset</t>
+          <t xml:space="preserve">Vehicle</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vehículo VENDIDO/entregado — relación cliente↔vehículo para posventa. Asset.Product2Id → Product2.</t>
+          <t xml:space="preserve">Inventario PROPIO de vehículos: cada unidad con VIN. Cadena: Vehicle.VehicleDefinitionId → VehicleDefinition; Vehicle.AssetId → Asset (que lleva el centro vía LocationId).</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">AccountId, Product2Id, SerialNumber=VIN, Status, PurchaseDate</t>
+          <t xml:space="preserve">Name, VehicleDefinitionId, VehicleIdentificationNumber (VIN — API name confirmado), AssetId, Status</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SerialNumber + AccountId</t>
+          <t xml:space="preserve">VehicleIdentificationNumber (único en la org)</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Histórico de ventas del DBM</t>
+          <t xml:space="preserve">Stock de vehículos del DBM (VLC) por centro</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Miles (histórico retroactivo)</t>
+          <t xml:space="preserve">DevSales: 6 hoy · miles al cargar · delta por movimiento</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">El flujo NUEVO ya lo crea solo (Order_Facturado_Handler al facturar). La carga aquí es únicamente el histórico anterior al go-live.</t>
+          <t xml:space="preserve">Cargar DESPUÉS del Asset (fila 9). Usados: entran por HU-045 (Appraisal → Vehicle). La búsqueda por centro filtra vía Asset.LocationId.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Plan de carga v4: reglas de kits provadas na org (Type=Bundle no pai, IsDefaultComponent=TRUE)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012ouMFEvRtMPEA2sZAxeatj
</commit_message>
<xml_diff>
--- a/docs/carga/Carga_Productos_Precios_Inventario.xlsx
+++ b/docs/carga/Carga_Productos_Precios_Inventario.xlsx
@@ -389,7 +389,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SapMaterialCode__c llega por el deploy (fila 0); backfill = MATNR también en los 250 existentes. Family distingue Vehículo / Repuesto / Accesorio (StandardValueSet Product2Family ya en el manifest).</t>
+          <t xml:space="preserve">SapMaterialCode__c llega por el deploy (fila 0); backfill = MATNR también en los 250 existentes. Family distingue Vehículo / Repuesto / Accesorio. REGLA DEL CATÁLOGO (probada 12/08): los productos que serán PADRE de kit deben cargarse con Type=Bundle.</t>
         </is>
       </c>
     </row>
@@ -552,12 +552,12 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DevSales: 0 hoy · centenas al cargar</t>
+          <t xml:space="preserve">DevSales: kit de prueba creado (SEED OK 12/08) · centenas al cargar</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Objeto habilitado y confirmado (12/08); ProductRelationshipTypeId = 0yoao0000019FldAAE en todos los registros.</t>
+          <t xml:space="preserve">REGLAS DEL CATÁLOGO probadas 12/08: ProductRelationshipTypeId = 0yoao0000019FldAAE (Bundle→BundleComponent), el padre con Type=Bundle (fila 3) e IsDefaultComponent=TRUE en cada componente (bundle estático).</t>
         </is>
       </c>
     </row>

</xml_diff>